<commit_message>
Fix emotional Stroop scoring: store corrAns and congruent as values
corrAns and congruent in trialTypes.xlsx were Excel formulas with no
cached results, so PsychoPy read them as empty and scored every emotional
Stroop response as incorrect (resp.corr = 0). Replace the formulas with the
values they compute: fearful face -> f, happy face -> h; congruent = 1 when
the face emotion matches the word. Data collected before this needs
rescoring from faceEmotion.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiment/task/trialTypes.xlsx
+++ b/experiment/task/trialTypes.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="trialTypes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="trialTypes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -932,13 +932,13 @@
           <t>../bw_image/bw_PS_0236.jpg</t>
         </is>
       </c>
-      <c r="D2">
-        <f>IF(B2="HAPPY", "h", IF(B2="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E2">
-        <f>IF(B2=A2, "1","0")</f>
-        <v/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -957,13 +957,13 @@
           <t>../bw_image/bw_KO_1082.jpg</t>
         </is>
       </c>
-      <c r="D3">
-        <f>IF(B3="HAPPY", "h", IF(B3="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E3">
-        <f>IF(B3=A3, "1","0")</f>
-        <v/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -982,13 +982,13 @@
           <t>../bw_image/bw_RA_3483.jpg</t>
         </is>
       </c>
-      <c r="D4">
-        <f>IF(B4="HAPPY", "h", IF(B4="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E4">
-        <f>IF(B4=A4, "1","0")</f>
-        <v/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1007,13 +1007,13 @@
           <t>../bw_image/bw_JS_0281.jpg</t>
         </is>
       </c>
-      <c r="D5">
-        <f>IF(B5="HAPPY", "h", IF(B5="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E5">
-        <f>IF(B5=A5, "1","0")</f>
-        <v/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
       </c>
       <c r="G5" s="1" t="n"/>
     </row>
@@ -1033,13 +1033,13 @@
           <t>../bw_image/bw_DC_0952.jpg</t>
         </is>
       </c>
-      <c r="D6">
-        <f>IF(B6="HAPPY", "h", IF(B6="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E6">
-        <f>IF(B6=A6, "1","0")</f>
-        <v/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
       </c>
       <c r="G6" s="1" t="n"/>
     </row>
@@ -1059,13 +1059,13 @@
           <t>../bw_image/bw_JG_0024.jpg</t>
         </is>
       </c>
-      <c r="D7">
-        <f>IF(B7="HAPPY", "h", IF(B7="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E7">
-        <f>IF(B7=A7, "1","0")</f>
-        <v/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
       </c>
       <c r="G7" s="1" t="n"/>
     </row>
@@ -1085,13 +1085,13 @@
           <t>../bw_image/bw_MJ_0271.jpg</t>
         </is>
       </c>
-      <c r="D8">
-        <f>IF(B8="HAPPY", "h", IF(B8="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E8">
-        <f>IF(B8=A8, "1","0")</f>
-        <v/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
       </c>
       <c r="G8" s="1" t="n"/>
     </row>
@@ -1111,13 +1111,13 @@
           <t>../bw_image/bw_MG_0330.jpg</t>
         </is>
       </c>
-      <c r="D9">
-        <f>IF(B9="HAPPY", "h", IF(B9="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E9">
-        <f>IF(B9=A9, "1","0")</f>
-        <v/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
       </c>
       <c r="G9" s="1" t="n"/>
     </row>
@@ -1137,13 +1137,13 @@
           <t>../bw_image/bw_MR1_1519.jpg</t>
         </is>
       </c>
-      <c r="D10">
-        <f>IF(B10="HAPPY", "h", IF(B10="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E10">
-        <f>IF(B10=A10, "1","0")</f>
-        <v/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
       </c>
       <c r="G10" s="1" t="n"/>
     </row>
@@ -1163,13 +1163,13 @@
           <t>../bw_image/bw_MK1_0746.jpg</t>
         </is>
       </c>
-      <c r="D11">
-        <f>IF(B11="HAPPY", "h", IF(B11="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E11">
-        <f>IF(B11=A11, "1","0")</f>
-        <v/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
       </c>
       <c r="G11" s="1" t="n"/>
     </row>
@@ -1189,13 +1189,13 @@
           <t>../bw_image/bw_KS_0624.jpg</t>
         </is>
       </c>
-      <c r="D12">
-        <f>IF(B12="HAPPY", "h", IF(B12="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E12">
-        <f>IF(B12=A12, "1","0")</f>
-        <v/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
       </c>
       <c r="G12" s="1" t="n"/>
     </row>
@@ -1215,13 +1215,13 @@
           <t>../bw_image/bw_JG_1465.jpg</t>
         </is>
       </c>
-      <c r="D13">
-        <f>IF(B13="HAPPY", "h", IF(B13="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E13">
-        <f>IF(B13=A13, "1","0")</f>
-        <v/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
       </c>
       <c r="G13" s="1" t="n"/>
     </row>
@@ -1241,13 +1241,13 @@
           <t>../bw_image/bw_KM_0137.jpg</t>
         </is>
       </c>
-      <c r="D14">
-        <f>IF(B14="HAPPY", "h", IF(B14="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E14">
-        <f>IF(B14=A14, "1","0")</f>
-        <v/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
       </c>
       <c r="G14" s="1" t="n"/>
     </row>
@@ -1267,13 +1267,13 @@
           <t>../bw_image/bw_MS_0291.jpg</t>
         </is>
       </c>
-      <c r="D15">
-        <f>IF(B15="HAPPY", "h", IF(B15="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E15">
-        <f>IF(B15=A15, "1","0")</f>
-        <v/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
       </c>
       <c r="G15" s="1" t="n"/>
     </row>
@@ -1293,13 +1293,13 @@
           <t>../bw_image/bw_MG_1280.jpg</t>
         </is>
       </c>
-      <c r="D16">
-        <f>IF(B16="HAPPY", "h", IF(B16="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E16">
-        <f>IF(B16=A16, "1","0")</f>
-        <v/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
       </c>
       <c r="G16" s="1" t="n"/>
     </row>
@@ -1319,13 +1319,13 @@
           <t>../bw_image/bw_MR1_0132.jpg</t>
         </is>
       </c>
-      <c r="D17">
-        <f>IF(B17="HAPPY", "h", IF(B17="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E17">
-        <f>IF(B17=A17, "1","0")</f>
-        <v/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
       </c>
       <c r="G17" s="1" t="n"/>
     </row>
@@ -1345,13 +1345,13 @@
           <t>../bw_image/bw_RA_0317.jpg</t>
         </is>
       </c>
-      <c r="D18">
-        <f>IF(B18="HAPPY", "h", IF(B18="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E18">
-        <f>IF(B18=A18, "1","0")</f>
-        <v/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
       </c>
       <c r="G18" s="1" t="n"/>
     </row>
@@ -1371,13 +1371,13 @@
           <t>../bw_image/bw_KA_0043.jpg</t>
         </is>
       </c>
-      <c r="D19">
-        <f>IF(B19="HAPPY", "h", IF(B19="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E19">
-        <f>IF(B19=A19, "1","0")</f>
-        <v/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
       </c>
       <c r="G19" s="1" t="n"/>
     </row>
@@ -1397,13 +1397,13 @@
           <t>../bw_image/bw_AG_0424.jpg</t>
         </is>
       </c>
-      <c r="D20">
-        <f>IF(B20="HAPPY", "h", IF(B20="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E20">
-        <f>IF(B20=A20, "1","0")</f>
-        <v/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
       <c r="G20" s="1" t="n"/>
     </row>
@@ -1423,13 +1423,13 @@
           <t>../bw_image/bw_PS_0157.jpg</t>
         </is>
       </c>
-      <c r="D21">
-        <f>IF(B21="HAPPY", "h", IF(B21="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E21">
-        <f>IF(B21=A21, "1","0")</f>
-        <v/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
       </c>
       <c r="G21" s="1" t="n"/>
     </row>
@@ -1449,13 +1449,13 @@
           <t>../bw_image/bw_AD_7950.jpg</t>
         </is>
       </c>
-      <c r="D22">
-        <f>IF(B22="HAPPY", "h", IF(B22="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E22">
-        <f>IF(B22=A22, "1","0")</f>
-        <v/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
       </c>
       <c r="G22" s="1" t="n"/>
     </row>
@@ -1475,13 +1475,13 @@
           <t>../bw_image/bw_RB_0392.jpg</t>
         </is>
       </c>
-      <c r="D23">
-        <f>IF(B23="HAPPY", "h", IF(B23="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E23">
-        <f>IF(B23=A23, "1","0")</f>
-        <v/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
       </c>
       <c r="G23" s="1" t="n"/>
     </row>
@@ -1501,13 +1501,13 @@
           <t>../bw_image/bw_SS_0018.jpg</t>
         </is>
       </c>
-      <c r="D24">
-        <f>IF(B24="HAPPY", "h", IF(B24="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E24">
-        <f>IF(B24=A24, "1","0")</f>
-        <v/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
       </c>
       <c r="G24" s="1" t="n"/>
     </row>
@@ -1527,13 +1527,13 @@
           <t>../bw_image/bw_JS_1601.jpg</t>
         </is>
       </c>
-      <c r="D25">
-        <f>IF(B25="HAPPY", "h", IF(B25="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E25">
-        <f>IF(B25=A25, "1","0")</f>
-        <v/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
       </c>
       <c r="G25" s="1" t="n"/>
     </row>
@@ -1553,13 +1553,13 @@
           <t>../bw_image/bw_PB_0499.jpg</t>
         </is>
       </c>
-      <c r="D26">
-        <f>IF(B26="HAPPY", "h", IF(B26="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E26">
-        <f>IF(B26=A26, "1","0")</f>
-        <v/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
       </c>
       <c r="G26" s="1" t="n"/>
     </row>
@@ -1579,13 +1579,13 @@
           <t>../bw_image/bw_SS_1188.jpg</t>
         </is>
       </c>
-      <c r="D27">
-        <f>IF(B27="HAPPY", "h", IF(B27="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E27">
-        <f>IF(B27=A27, "1","0")</f>
-        <v/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
       </c>
       <c r="G27" s="1" t="n"/>
     </row>
@@ -1605,13 +1605,13 @@
           <t>../bw_image/bw_AG_0086.jpg</t>
         </is>
       </c>
-      <c r="D28">
-        <f>IF(B28="HAPPY", "h", IF(B28="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E28">
-        <f>IF(B28=A28, "1","0")</f>
-        <v/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
       </c>
       <c r="G28" s="1" t="n"/>
     </row>
@@ -1631,13 +1631,13 @@
           <t>../bw_image/bw_SO_1515.jpg</t>
         </is>
       </c>
-      <c r="D29">
-        <f>IF(B29="HAPPY", "h", IF(B29="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E29">
-        <f>IF(B29=A29, "1","0")</f>
-        <v/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
       </c>
       <c r="G29" s="1" t="n"/>
     </row>
@@ -1657,13 +1657,13 @@
           <t>../bw_image/bw_MB_1031.jpg</t>
         </is>
       </c>
-      <c r="D30">
-        <f>IF(B30="HAPPY", "h", IF(B30="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E30">
-        <f>IF(B30=A30, "1","0")</f>
-        <v/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
       </c>
       <c r="G30" s="1" t="n"/>
     </row>
@@ -1683,13 +1683,13 @@
           <t>../bw_image/bw_MR_0959.jpg</t>
         </is>
       </c>
-      <c r="D31">
-        <f>IF(B31="HAPPY", "h", IF(B31="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E31">
-        <f>IF(B31=A31, "1","0")</f>
-        <v/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
       </c>
       <c r="G31" s="1" t="n"/>
     </row>
@@ -1709,13 +1709,13 @@
           <t>../bw_image/bw_KO_0277.jpg</t>
         </is>
       </c>
-      <c r="D32">
-        <f>IF(B32="HAPPY", "h", IF(B32="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E32">
-        <f>IF(B32=A32, "1","0")</f>
-        <v/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
       </c>
       <c r="G32" s="1" t="n"/>
     </row>
@@ -1735,13 +1735,13 @@
           <t>../bw_image/bw_KS_4222.jpg</t>
         </is>
       </c>
-      <c r="D33">
-        <f>IF(B33="HAPPY", "h", IF(B33="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E33">
-        <f>IF(B33=A33, "1","0")</f>
-        <v/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
       </c>
       <c r="G33" s="1" t="n"/>
     </row>
@@ -1761,13 +1761,13 @@
           <t>../bw_image/bw_KL_0092.jpg</t>
         </is>
       </c>
-      <c r="D34">
-        <f>IF(B34="HAPPY", "h", IF(B34="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E34">
-        <f>IF(B34=A34, "1","0")</f>
-        <v/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
       </c>
       <c r="G34" s="1" t="n"/>
     </row>
@@ -1787,13 +1787,13 @@
           <t>../bw_image/bw_KP_1148.jpg</t>
         </is>
       </c>
-      <c r="D35">
-        <f>IF(B35="HAPPY", "h", IF(B35="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E35">
-        <f>IF(B35=A35, "1","0")</f>
-        <v/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
       </c>
       <c r="G35" s="1" t="n"/>
     </row>
@@ -1813,13 +1813,13 @@
           <t>../bw_image/bw_DC_0139.jpg</t>
         </is>
       </c>
-      <c r="D36">
-        <f>IF(B36="HAPPY", "h", IF(B36="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E36">
-        <f>IF(B36=A36, "1","0")</f>
-        <v/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
       </c>
       <c r="G36" s="1" t="n"/>
     </row>
@@ -1839,13 +1839,13 @@
           <t>../bw_image/bw_KM_1980.jpg</t>
         </is>
       </c>
-      <c r="D37">
-        <f>IF(B37="HAPPY", "h", IF(B37="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E37">
-        <f>IF(B37=A37, "1","0")</f>
-        <v/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
       </c>
       <c r="G37" s="1" t="n"/>
     </row>
@@ -1865,13 +1865,13 @@
           <t>../bw_image/bw_KL_0900.jpg</t>
         </is>
       </c>
-      <c r="D38">
-        <f>IF(B38="HAPPY", "h", IF(B38="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E38">
-        <f>IF(B38=A38, "1","0")</f>
-        <v/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
       </c>
       <c r="G38" s="1" t="n"/>
     </row>
@@ -1891,13 +1891,13 @@
           <t>../bw_image/bw_MR_0055.jpg</t>
         </is>
       </c>
-      <c r="D39">
-        <f>IF(B39="HAPPY", "h", IF(B39="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E39">
-        <f>IF(B39=A39, "1","0")</f>
-        <v/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
       </c>
       <c r="G39" s="1" t="n"/>
     </row>
@@ -1917,13 +1917,13 @@
           <t>../bw_image/bw_KA_1134.jpg</t>
         </is>
       </c>
-      <c r="D40">
-        <f>IF(B40="HAPPY", "h", IF(B40="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E40">
-        <f>IF(B40=A40, "1","0")</f>
-        <v/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
       </c>
       <c r="G40" s="1" t="n"/>
     </row>
@@ -1943,13 +1943,13 @@
           <t>../bw_image/bw_MK_0364.jpg</t>
         </is>
       </c>
-      <c r="D41">
-        <f>IF(B41="HAPPY", "h", IF(B41="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E41">
-        <f>IF(B41=A41, "1","0")</f>
-        <v/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
       </c>
       <c r="G41" s="1" t="n"/>
     </row>
@@ -1969,13 +1969,13 @@
           <t>../bw_image/bw_KP_0051.jpg</t>
         </is>
       </c>
-      <c r="D42">
-        <f>IF(B42="HAPPY", "h", IF(B42="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E42">
-        <f>IF(B42=A42, "1","0")</f>
-        <v/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
       </c>
       <c r="G42" s="1" t="n"/>
     </row>
@@ -1995,13 +1995,13 @@
           <t>../bw_image/bw_MR2_0063.jpg</t>
         </is>
       </c>
-      <c r="D43">
-        <f>IF(B43="HAPPY", "h", IF(B43="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E43">
-        <f>IF(B43=A43, "1","0")</f>
-        <v/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
       </c>
       <c r="G43" s="1" t="n"/>
     </row>
@@ -2021,13 +2021,13 @@
           <t>../bw_image/bw_SO_0028.jpg</t>
         </is>
       </c>
-      <c r="D44">
-        <f>IF(B44="HAPPY", "h", IF(B44="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E44">
-        <f>IF(B44=A44, "1","0")</f>
-        <v/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
       </c>
       <c r="G44" s="1" t="n"/>
     </row>
@@ -2047,13 +2047,13 @@
           <t>../bw_image/bw_PB_0269.jpg</t>
         </is>
       </c>
-      <c r="D45">
-        <f>IF(B45="HAPPY", "h", IF(B45="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E45">
-        <f>IF(B45=A45, "1","0")</f>
-        <v/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
       </c>
       <c r="G45" s="1" t="n"/>
     </row>
@@ -2073,13 +2073,13 @@
           <t>../bw_image/bw_PA_0394.jpg</t>
         </is>
       </c>
-      <c r="D46">
-        <f>IF(B46="HAPPY", "h", IF(B46="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E46">
-        <f>IF(B46=A46, "1","0")</f>
-        <v/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
       </c>
       <c r="G46" s="1" t="n"/>
     </row>
@@ -2099,13 +2099,13 @@
           <t>../bw_image/bw_PO_0124.jpg</t>
         </is>
       </c>
-      <c r="D47">
-        <f>IF(B47="HAPPY", "h", IF(B47="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E47">
-        <f>IF(B47=A47, "1","0")</f>
-        <v/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
       </c>
       <c r="G47" s="1" t="n"/>
     </row>
@@ -2125,13 +2125,13 @@
           <t>../bw_image/bw_PA_0112.jpg</t>
         </is>
       </c>
-      <c r="D48">
-        <f>IF(B48="HAPPY", "h", IF(B48="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E48">
-        <f>IF(B48=A48, "1","0")</f>
-        <v/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
       </c>
       <c r="G48" s="1" t="n"/>
     </row>
@@ -2151,13 +2151,13 @@
           <t>../bw_image/bw_MJ_0066.jpg</t>
         </is>
       </c>
-      <c r="D49">
-        <f>IF(B49="HAPPY", "h", IF(B49="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E49">
-        <f>IF(B49=A49, "1","0")</f>
-        <v/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
       </c>
       <c r="G49" s="1" t="n"/>
     </row>
@@ -2177,13 +2177,13 @@
           <t>../bw_image/bw_MK1_0087.jpg</t>
         </is>
       </c>
-      <c r="D50">
-        <f>IF(B50="HAPPY", "h", IF(B50="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E50">
-        <f>IF(B50=A50, "1","0")</f>
-        <v/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
       </c>
       <c r="G50" s="1" t="n"/>
     </row>
@@ -2203,13 +2203,13 @@
           <t>../bw_image/bw_MR2_1829.jpg</t>
         </is>
       </c>
-      <c r="D51">
-        <f>IF(B51="HAPPY", "h", IF(B51="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E51">
-        <f>IF(B51=A51, "1","0")</f>
-        <v/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
       </c>
       <c r="G51" s="1" t="n"/>
     </row>
@@ -2229,13 +2229,13 @@
           <t>../bw_image/bw_HW_0068.jpg</t>
         </is>
       </c>
-      <c r="D52">
-        <f>IF(B52="HAPPY", "h", IF(B52="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E52">
-        <f>IF(B52=A52, "1","0")</f>
-        <v/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
       </c>
       <c r="G52" s="1" t="n"/>
     </row>
@@ -2255,13 +2255,13 @@
           <t>../bw_image/bw_AD_8432.jpg</t>
         </is>
       </c>
-      <c r="D53">
-        <f>IF(B53="HAPPY", "h", IF(B53="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E53">
-        <f>IF(B53=A53, "1","0")</f>
-        <v/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
       </c>
       <c r="G53" s="1" t="n"/>
     </row>
@@ -2281,13 +2281,13 @@
           <t>../bw_image/bw_OG_6189.jpg</t>
         </is>
       </c>
-      <c r="D54">
-        <f>IF(B54="HAPPY", "h", IF(B54="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E54">
-        <f>IF(B54=A54, "1","0")</f>
-        <v/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
       </c>
       <c r="G54" s="1" t="n"/>
     </row>
@@ -2307,13 +2307,13 @@
           <t>../bw_image/bw_HW_2219.jpg</t>
         </is>
       </c>
-      <c r="D55">
-        <f>IF(B55="HAPPY", "h", IF(B55="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E55">
-        <f>IF(B55=A55, "1","0")</f>
-        <v/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
       </c>
       <c r="G55" s="1" t="n"/>
     </row>
@@ -2333,13 +2333,13 @@
           <t>../bw_image/bw_RB_0329.jpg</t>
         </is>
       </c>
-      <c r="D56">
-        <f>IF(B56="HAPPY", "h", IF(B56="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E56">
-        <f>IF(B56=A56, "1","0")</f>
-        <v/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
       </c>
       <c r="G56" s="1" t="n"/>
     </row>
@@ -2359,13 +2359,13 @@
           <t>../bw_image/bw_MB_0048.jpg</t>
         </is>
       </c>
-      <c r="D57">
-        <f>IF(B57="HAPPY", "h", IF(B57="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E57">
-        <f>IF(B57=A57, "1","0")</f>
-        <v/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
       </c>
       <c r="G57" s="1" t="n"/>
     </row>
@@ -2385,13 +2385,13 @@
           <t>../bw_image/bw_PO_1030.jpg</t>
         </is>
       </c>
-      <c r="D58">
-        <f>IF(B58="HAPPY", "h", IF(B58="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E58">
-        <f>IF(B58=A58, "1","0")</f>
-        <v/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
       </c>
       <c r="G58" s="1" t="n"/>
     </row>
@@ -2411,13 +2411,13 @@
           <t>../bw_image/bw_MS_0226.jpg</t>
         </is>
       </c>
-      <c r="D59">
-        <f>IF(B59="HAPPY", "h", IF(B59="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E59">
-        <f>IF(B59=A59, "1","0")</f>
-        <v/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
       </c>
       <c r="G59" s="1" t="n"/>
     </row>
@@ -2437,13 +2437,13 @@
           <t>../bw_image/bw_OG_7620.jpg</t>
         </is>
       </c>
-      <c r="D60">
-        <f>IF(B60="HAPPY", "h", IF(B60="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E60">
-        <f>IF(B60=A60, "1","0")</f>
-        <v/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
       </c>
       <c r="G60" s="1" t="n"/>
     </row>
@@ -2463,13 +2463,13 @@
           <t>../bw_image/bw_MK_0040.jpg</t>
         </is>
       </c>
-      <c r="D61">
-        <f>IF(B61="HAPPY", "h", IF(B61="FEAR", "f", ""))</f>
-        <v/>
-      </c>
-      <c r="E61">
-        <f>IF(B61=A61, "1","0")</f>
-        <v/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
       </c>
       <c r="G61" s="1" t="n"/>
     </row>

</xml_diff>